<commit_message>
clean: vaciar TODOS los datos transaccionales del dashboard
Vaciados (solo cabeceras para que no crashee):
- F&B: ventas_fb_diarias, pos_ventas, pos_ordenes, inventario, mermas, recetas
- AR OTAs: facturas_ota_demo
- AR Real: clientes_credito, reservas_credito, rooming_demo
- Banco: extracto_banco
- Notificaciones: historial vacío
- Archivos procesados: JSON vacío

Preservados (configuración):
- proveedores.xlsx, plan_cuentas.xlsx, comisiones_pactadas.xlsx
- kpis_hoteles.xlsx (datos Calipolis para demo)
- hotel_config.json, hoteles.json, usuarios.json

Ahora el dashboard está completamente vacío — cada tab mostrará
'Sin datos' hasta que el usuario suba archivos con ⚡ Procesar Archivos.
</commit_message>
<xml_diff>
--- a/datos-referencia/recetas.xlsx
+++ b/datos-referencia/recetas.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recetas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,283 +413,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>id_receta</t>
+          <t>plato</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>nombre</t>
+          <t>ingrediente</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>categoria</t>
+          <t>cantidad</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>precio_venta</t>
+          <t>unidad</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>ingredientes_json</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>REC001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paella de Marisco</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Arroces</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>[{"ingrediente":"Arroz","cantidad":0.15,"unidad":"kg","coste_unitario":1.20},{"ingrediente":"Gambas","cantidad":0.12,"unidad":"kg","coste_unitario":12.00},{"ingrediente":"Mejillones","cantidad":0.10,"unidad":"kg","coste_unitario":4.50},{"ingrediente":"Caldo Pescado","cantidad":0.30,"unidad":"l","coste_unitario":0.80},{"ingrediente":"Aceite Oliva","cantidad":0.02,"unidad":"l","coste_unitario":3.50}]</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>REC002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Chuletón de Ternera</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Carnes</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>32</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>[{"ingrediente":"Ternera Chuleton","cantidad":0.35,"unidad":"kg","coste_unitario":22.00},{"ingrediente":"Patatas","cantidad":0.20,"unidad":"kg","coste_unitario":0.60},{"ingrediente":"Sal","cantidad":0.005,"unidad":"kg","coste_unitario":0.50},{"ingrediente":"Aceite Oliva","cantidad":0.01,"unidad":"l","coste_unitario":3.50}]</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>REC003</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Gazpacho</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Sopas Frías</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>[{"ingrediente":"Tomate","cantidad":0.30,"unidad":"kg","coste_unitario":1.80},{"ingrediente":"Pepino","cantidad":0.05,"unidad":"kg","coste_unitario":1.20},{"ingrediente":"Pimiento","cantidad":0.04,"unidad":"kg","coste_unitario":1.50},{"ingrediente":"Pan","cantidad":0.03,"unidad":"kg","coste_unitario":2.00},{"ingrediente":"Aceite Oliva","cantidad":0.02,"unidad":"l","coste_unitario":3.50}]</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>REC004</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Crema Catalana</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Postres</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>[{"ingrediente":"Nata","cantidad":0.15,"unidad":"l","coste_unitario":2.20},{"ingrediente":"Leche","cantidad":0.10,"unidad":"l","coste_unitario":0.90},{"ingrediente":"Huevos","cantidad":0.10,"unidad":"kg","coste_unitario":2.80},{"ingrediente":"Azucar","cantidad":0.04,"unidad":"kg","coste_unitario":1.10}]</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>REC005</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Gin Tonic Premium</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Bebidas</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>12</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>[{"ingrediente":"Ginebra Premium","cantidad":0.05,"unidad":"l","coste_unitario":28.00},{"ingrediente":"Tonica","cantidad":0.20,"unidad":"l","coste_unitario":1.80},{"ingrediente":"Limon","cantidad":0.02,"unidad":"kg","coste_unitario":1.50}]</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>REC006</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Ensalada César</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Ensaladas</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>[{"ingrediente":"Lechuga","cantidad":0.12,"unidad":"kg","coste_unitario":1.40},{"ingrediente":"Pollo","cantidad":0.10,"unidad":"kg","coste_unitario":6.50},{"ingrediente":"Parmesano","cantidad":0.03,"unidad":"kg","coste_unitario":18.00},{"ingrediente":"Pan","cantidad":0.04,"unidad":"kg","coste_unitario":2.00}]</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>REC007</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Lubina a la Sal</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Pescados</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>28</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>[{"ingrediente":"Lubina","cantidad":0.40,"unidad":"kg","coste_unitario":14.00},{"ingrediente":"Sal Gorda","cantidad":0.50,"unidad":"kg","coste_unitario":0.40},{"ingrediente":"Aceite Oliva","cantidad":0.02,"unidad":"l","coste_unitario":3.50}]</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>REC008</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Tarta de Queso</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Postres</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>[{"ingrediente":"Queso Crema","cantidad":0.15,"unidad":"kg","coste_unitario":5.50},{"ingrediente":"Nata","cantidad":0.08,"unidad":"l","coste_unitario":2.20},{"ingrediente":"Huevos","cantidad":0.06,"unidad":"kg","coste_unitario":2.80},{"ingrediente":"Azucar","cantidad":0.05,"unidad":"kg","coste_unitario":1.10},{"ingrediente":"Galletas","cantidad":0.06,"unidad":"kg","coste_unitario":3.20}]</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>REC009</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Vino Tinto Copa</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Bebidas</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>[{"ingrediente":"Vino Tinto","cantidad":0.15,"unidad":"l","coste_unitario":6.00}]</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>REC010</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Agua Mineral</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Bebidas</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>[{"ingrediente":"Agua Mineral","cantidad":0.50,"unidad":"l","coste_unitario":0.35}]</t>
+          <t>coste_kg</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>coste_total</t>
         </is>
       </c>
     </row>

</xml_diff>